<commit_message>
few  changes in the SAP
</commit_message>
<xml_diff>
--- a/pages/SAP/BP Test Data.xlsx
+++ b/pages/SAP/BP Test Data.xlsx
@@ -8,20 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\pages\SAP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52D1CEE8-DE59-4BE1-91A3-8629AA754D5C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{714216D2-33F1-4393-A8F1-CB830CFCAA4E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PC" sheetId="1" r:id="rId1"/>
     <sheet name="MC" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PC!$A$1:$C$72</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="358">
   <si>
     <t>PC</t>
   </si>
@@ -464,48 +467,72 @@
     <t>781031-12-5549</t>
   </si>
   <si>
+    <t>1000027600</t>
+  </si>
+  <si>
     <t>JFG8942</t>
   </si>
   <si>
     <t>691129-01-5381</t>
   </si>
   <si>
+    <t>1000017149</t>
+  </si>
+  <si>
     <t>JNP4438</t>
   </si>
   <si>
     <t>990915-01-5178</t>
   </si>
   <si>
+    <t>1000018557</t>
+  </si>
+  <si>
     <t>WTH8270</t>
   </si>
   <si>
     <t>860927-33-5739</t>
   </si>
   <si>
+    <t>1000017716</t>
+  </si>
+  <si>
     <t>AJG6911</t>
   </si>
   <si>
     <t>790618-08-6264</t>
   </si>
   <si>
+    <t>1000016150</t>
+  </si>
+  <si>
     <t>CCK4009</t>
   </si>
   <si>
     <t>830129-06-5239</t>
   </si>
   <si>
+    <t>1000016230</t>
+  </si>
+  <si>
     <t>WXA267</t>
   </si>
   <si>
     <t>000731-01-0019</t>
   </si>
   <si>
+    <t>1000017108</t>
+  </si>
+  <si>
     <t>JLN6674</t>
   </si>
   <si>
     <t>411028-01-5009</t>
   </si>
   <si>
+    <t>1000017733</t>
+  </si>
+  <si>
     <t>WWP9818</t>
   </si>
   <si>
@@ -758,12 +785,18 @@
     <t>990730-04-5119</t>
   </si>
   <si>
+    <t>1000017882</t>
+  </si>
+  <si>
     <t>JUP7861</t>
   </si>
   <si>
     <t>040711-01-0405</t>
   </si>
   <si>
+    <t>1000017109</t>
+  </si>
+  <si>
     <t>JMD9586</t>
   </si>
   <si>
@@ -1062,6 +1095,9 @@
   </si>
   <si>
     <t>001209-11-0169</t>
+  </si>
+  <si>
+    <t>BP</t>
   </si>
 </sst>
 </file>
@@ -1154,12 +1190,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1493,11 +1532,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="5"/>
-      <c r="C1" s="6"/>
+      <c r="C1" s="4" t="s">
+        <v>357</v>
+      </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
@@ -2067,176 +2108,192 @@
       <c r="B53" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="C53" s="2"/>
+      <c r="C53" s="2" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="C54" s="2"/>
+        <v>149</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>150</v>
+      </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" s="1" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="C55" s="2"/>
+        <v>152</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>153</v>
+      </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="C56" s="2"/>
+        <v>155</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" s="1" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="C57" s="2"/>
+        <v>158</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" s="1" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="C58" s="2"/>
+        <v>161</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>162</v>
+      </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" s="1" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="C59" s="2"/>
+        <v>164</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" s="1" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="C60" s="2"/>
+        <v>167</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>168</v>
+      </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" s="1" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="C61" s="2"/>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" s="1" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="C62" s="2"/>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" s="1" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="C63" s="2"/>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" s="1" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="C64" s="2"/>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" s="1" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="C65" s="2"/>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" s="1" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="C66" s="2"/>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" s="1" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="C67" s="2"/>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" s="1" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="C68" s="2"/>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" s="1" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="C69" s="2"/>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" s="1" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="C70" s="2"/>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" s="1" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="C71" s="2"/>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" s="1" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="C72" s="2"/>
     </row>
@@ -2319,8 +2376,11 @@
       <c r="C98" s="2"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C72" xr:uid="{5D2E8815-BE8F-4B1C-94FF-B221273C007B}">
+    <filterColumn colId="0" showButton="0"/>
+  </autoFilter>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -2338,686 +2398,696 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="6"/>
+      <c r="A1" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="7"/>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="1" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="1" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="1" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="1" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="1" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="1" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="1" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="1" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="1" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="1" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="1" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" s="1" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="1" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="1" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="1" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="1" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="1" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>244</v>
-      </c>
-      <c r="C21" s="2"/>
+        <v>252</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>253</v>
+      </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="1" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="C22" s="2"/>
+        <v>255</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="1" t="s">
-        <v>247</v>
+        <v>257</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="C23" s="2"/>
+        <v>258</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="1" t="s">
-        <v>249</v>
+        <v>259</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>250</v>
-      </c>
-      <c r="C24" s="2"/>
+        <v>260</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="1" t="s">
-        <v>251</v>
+        <v>261</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>252</v>
-      </c>
-      <c r="C25" s="2"/>
+        <v>262</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" s="1" t="s">
-        <v>253</v>
+        <v>263</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>254</v>
+        <v>264</v>
       </c>
       <c r="C26" s="2"/>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="1" t="s">
-        <v>255</v>
+        <v>265</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>256</v>
+        <v>266</v>
       </c>
       <c r="C27" s="2"/>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" s="1" t="s">
-        <v>257</v>
+        <v>267</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>258</v>
+        <v>268</v>
       </c>
       <c r="C28" s="2"/>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" s="1" t="s">
-        <v>259</v>
+        <v>269</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="C29" s="2"/>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" s="1" t="s">
-        <v>261</v>
+        <v>271</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>262</v>
+        <v>272</v>
       </c>
       <c r="C30" s="2"/>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" s="1" t="s">
-        <v>263</v>
+        <v>273</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>264</v>
+        <v>274</v>
       </c>
       <c r="C31" s="2"/>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" s="1" t="s">
-        <v>265</v>
+        <v>275</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>266</v>
+        <v>276</v>
       </c>
       <c r="C32" s="2"/>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" s="1" t="s">
-        <v>267</v>
+        <v>277</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>268</v>
+        <v>278</v>
       </c>
       <c r="C33" s="2"/>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" s="1" t="s">
-        <v>269</v>
+        <v>279</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>270</v>
+        <v>280</v>
       </c>
       <c r="C34" s="2"/>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" s="1" t="s">
-        <v>271</v>
+        <v>281</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>272</v>
+        <v>282</v>
       </c>
       <c r="C35" s="2"/>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" s="1" t="s">
-        <v>273</v>
+        <v>283</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>274</v>
+        <v>284</v>
       </c>
       <c r="C36" s="2"/>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" s="1" t="s">
-        <v>275</v>
+        <v>285</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>276</v>
+        <v>286</v>
       </c>
       <c r="C37" s="2"/>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" s="1" t="s">
-        <v>277</v>
+        <v>287</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>278</v>
+        <v>288</v>
       </c>
       <c r="C38" s="2"/>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" s="1" t="s">
-        <v>279</v>
+        <v>289</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>280</v>
+        <v>290</v>
       </c>
       <c r="C39" s="2"/>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" s="1" t="s">
-        <v>281</v>
+        <v>291</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>282</v>
+        <v>292</v>
       </c>
       <c r="C40" s="2"/>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" s="1" t="s">
-        <v>283</v>
+        <v>293</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>284</v>
+        <v>294</v>
       </c>
       <c r="C41" s="2"/>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" s="1" t="s">
-        <v>285</v>
+        <v>295</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>286</v>
+        <v>296</v>
       </c>
       <c r="C42" s="2"/>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" s="1" t="s">
-        <v>287</v>
+        <v>297</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>288</v>
+        <v>298</v>
       </c>
       <c r="C43" s="2"/>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" s="1" t="s">
-        <v>289</v>
+        <v>299</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="C44" s="2"/>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" s="1" t="s">
-        <v>291</v>
+        <v>301</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>292</v>
+        <v>302</v>
       </c>
       <c r="C45" s="2"/>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" s="1" t="s">
-        <v>293</v>
+        <v>303</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>294</v>
+        <v>304</v>
       </c>
       <c r="C46" s="2"/>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" s="1" t="s">
-        <v>295</v>
+        <v>305</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>296</v>
+        <v>306</v>
       </c>
       <c r="C47" s="2"/>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" s="1" t="s">
-        <v>297</v>
+        <v>307</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>298</v>
+        <v>308</v>
       </c>
       <c r="C48" s="2"/>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" s="1" t="s">
-        <v>299</v>
+        <v>309</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>300</v>
+        <v>310</v>
       </c>
       <c r="C49" s="2"/>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" s="1" t="s">
-        <v>301</v>
+        <v>311</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>302</v>
+        <v>312</v>
       </c>
       <c r="C50" s="2"/>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" s="1" t="s">
-        <v>303</v>
+        <v>313</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>304</v>
+        <v>314</v>
       </c>
       <c r="C51" s="2"/>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" s="1" t="s">
-        <v>305</v>
+        <v>315</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>306</v>
+        <v>316</v>
       </c>
       <c r="C52" s="2"/>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" s="1" t="s">
-        <v>307</v>
+        <v>317</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>308</v>
+        <v>318</v>
       </c>
       <c r="C53" s="2"/>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" s="1" t="s">
-        <v>309</v>
+        <v>319</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>310</v>
+        <v>320</v>
       </c>
       <c r="C54" s="2"/>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" s="1" t="s">
-        <v>311</v>
+        <v>321</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>312</v>
+        <v>322</v>
       </c>
       <c r="C55" s="2"/>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" s="1" t="s">
-        <v>313</v>
+        <v>323</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>314</v>
+        <v>324</v>
       </c>
       <c r="C56" s="2"/>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" s="1" t="s">
-        <v>315</v>
+        <v>325</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>316</v>
+        <v>326</v>
       </c>
       <c r="C57" s="2"/>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" s="1" t="s">
-        <v>317</v>
+        <v>327</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>318</v>
+        <v>328</v>
       </c>
       <c r="C58" s="2"/>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" s="1" t="s">
-        <v>319</v>
+        <v>329</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>320</v>
+        <v>330</v>
       </c>
       <c r="C59" s="2"/>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" s="1" t="s">
-        <v>321</v>
+        <v>331</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>322</v>
+        <v>332</v>
       </c>
       <c r="C60" s="2"/>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" s="1" t="s">
-        <v>323</v>
+        <v>333</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>324</v>
+        <v>334</v>
       </c>
       <c r="C61" s="2"/>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" s="1" t="s">
-        <v>325</v>
+        <v>335</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>326</v>
+        <v>336</v>
       </c>
       <c r="C62" s="2"/>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" s="1" t="s">
-        <v>327</v>
+        <v>337</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>328</v>
+        <v>338</v>
       </c>
       <c r="C63" s="2"/>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" s="1" t="s">
-        <v>329</v>
+        <v>339</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>330</v>
+        <v>340</v>
       </c>
       <c r="C64" s="2"/>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" s="1" t="s">
-        <v>331</v>
+        <v>341</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="C65" s="2"/>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" s="1" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>334</v>
+        <v>344</v>
       </c>
       <c r="C66" s="2"/>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" s="1" t="s">
-        <v>335</v>
+        <v>345</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>336</v>
+        <v>346</v>
       </c>
       <c r="C67" s="2"/>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" s="1" t="s">
-        <v>337</v>
+        <v>347</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>338</v>
+        <v>348</v>
       </c>
       <c r="C68" s="2"/>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" s="1" t="s">
-        <v>339</v>
+        <v>349</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>340</v>
+        <v>350</v>
       </c>
       <c r="C69" s="2"/>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" s="1" t="s">
-        <v>341</v>
+        <v>351</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>342</v>
+        <v>352</v>
       </c>
       <c r="C70" s="2"/>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" s="1" t="s">
-        <v>343</v>
+        <v>353</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>344</v>
+        <v>354</v>
       </c>
       <c r="C71" s="2"/>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" s="1" t="s">
-        <v>345</v>
+        <v>355</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>346</v>
+        <v>356</v>
       </c>
       <c r="C72" s="2"/>
     </row>

</xml_diff>